<commit_message>
Rename Excel 'Pay Notes' sheet to 'Pay Guide'
Renames the workbook tab (and its print-area/print-title references) and
the two in-sheet mentions that point readers to it, done via direct XML
edit so all formatting, formulas and protection are preserved untouched.
Also updates the workbook description on the calculator page.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FxBSYkNTAwxShAqXto2QT4
</commit_message>
<xml_diff>
--- a/PayCalc_V19.xlsx
+++ b/PayCalc_V19.xlsx
@@ -9,15 +9,15 @@
   </bookViews>
   <sheets>
     <sheet name="Pay Calculator" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Pay Notes" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Pay Guide" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Settings &amp; Rates" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Tax Engine" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Pay Calculator'!$A$1:$J$99</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Pay Calculator'!$1:$2</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Pay Notes'!$A$1:$J$51</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'Pay Notes'!$1:$2</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Pay Guide'!$A$1:$J$51</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'Pay Guide'!$1:$2</definedName>
     <definedName function="false" hidden="false" name="BaseRate" vbProcedure="false">'Tax Engine'!$F$5</definedName>
     <definedName function="false" hidden="false" name="ConcCap" vbProcedure="false">'Settings &amp; Rates'!$B$44</definedName>
     <definedName function="false" hidden="false" name="ContribTax" vbProcedure="false">'Settings &amp; Rates'!$B$42</definedName>
@@ -528,7 +528,7 @@
     <t xml:space="preserve">Leave the payslip column blank when you are not reconciling. A mismatch usually means a rate on Settings &amp; Rates is stale, or payroll treats an allowance differently — see block E for the clause each rate comes from.</t>
   </si>
   <si>
-    <t xml:space="preserve">PayCalc V19 · pay scale award 01.09.2025 · tax tables ATO 01.07.2026 · plain-English guide on the Pay Notes tab · rates, sources &amp; incoming changes on Settings &amp; Rates</t>
+    <t xml:space="preserve">PayCalc V19 · pay scale award 01.09.2025 · tax tables ATO 01.07.2026 · plain-English guide on the Pay Guide tab · rates, sources &amp; incoming changes on Settings &amp; Rates</t>
   </si>
   <si>
     <t xml:space="preserve">PAY  NOTES</t>
@@ -1023,7 +1023,7 @@
     <t xml:space="preserve">OFFER 16.07.2026 — not yet certified</t>
   </si>
   <si>
-    <t xml:space="preserve">Employer Offer dated 16.07.2026 (3-year term, expires 31.07.2029). Three increases: 1 Aug 2026 = 3.5% (3% + 0.5% CPI uplift, already triggered), 1 Aug 2027 = 2.5%, 1 Aug 2028 = 2.5%. The FIRST rise applies to the higher of Award or Agreement — i.e. the Award rate (cl 2.18(6) retained). Allowances that track wages rise by the same %. CONDITIONAL: all unions must agree in-principle by 31.08.2026 to hold the 1 Aug date, else it shifts to the first of the month agreement is reached. NOT applied yet — do not change rates until certified. When certified, the EBA rise builds a SEPARATE agreement ladder — it must NOT be added to block A. Block A is the AWARD ladder; it moves only at a State Wage Case / reprint (~1 Sep). The certification (~1 Aug) and the SWC (~1 Sep) are only 31 days apart, so bumping block A on certification would be overwritten a month later = double-bump. Correct method: 1) build an Agreement-rate column = (award rate at 31.07.2026) × the agreed % for each row; 2) operational rate + $379 cap × same %; 3) set pay = MAX(award, agreement) per row (cl 2.18(6)); 4) block A itself changes ONLY at the SWC/reprint; 5) pull the Rates-checked-until tripwire back to the first-rise date (1 Aug if unions agree by 31 Aug); 6) footer date. Do NOT index: retention (cl 2.12(5) — not subject to annual increase, stays $45.00), shift % (a % of earnings — self-indexes; only change if the certified % changes), qualification (cl 4.2 — no indexation clause, hold pending certified text), in-charge/laundry (move with the award/SWC, not the EBA). YEARS 2-3: each 1 Aug, agreement ladder × 1.025 applied to the PRECEDING AGREEMENT rate (offer wording), NOT the award. After each 1 Sep SWC the award ladder moves independently — keep BOTH ladders live and re-check the MAX winner per row. Caution: if an SWC is ever a flat dollar amount or tiered (not a flat %), the winning ladder can differ by classification — don't assume a blanket MAX. If certification lands after 1 Aug, the first rise backdates and arrives lump-sum-taxed — use the 'Other taxable earnings' row and point to the Pay Notes lump-sum explainer.</t>
+    <t xml:space="preserve">Employer Offer dated 16.07.2026 (3-year term, expires 31.07.2029). Three increases: 1 Aug 2026 = 3.5% (3% + 0.5% CPI uplift, already triggered), 1 Aug 2027 = 2.5%, 1 Aug 2028 = 2.5%. The FIRST rise applies to the higher of Award or Agreement — i.e. the Award rate (cl 2.18(6) retained). Allowances that track wages rise by the same %. CONDITIONAL: all unions must agree in-principle by 31.08.2026 to hold the 1 Aug date, else it shifts to the first of the month agreement is reached. NOT applied yet — do not change rates until certified. When certified, the EBA rise builds a SEPARATE agreement ladder — it must NOT be added to block A. Block A is the AWARD ladder; it moves only at a State Wage Case / reprint (~1 Sep). The certification (~1 Aug) and the SWC (~1 Sep) are only 31 days apart, so bumping block A on certification would be overwritten a month later = double-bump. Correct method: 1) build an Agreement-rate column = (award rate at 31.07.2026) × the agreed % for each row; 2) operational rate + $379 cap × same %; 3) set pay = MAX(award, agreement) per row (cl 2.18(6)); 4) block A itself changes ONLY at the SWC/reprint; 5) pull the Rates-checked-until tripwire back to the first-rise date (1 Aug if unions agree by 31 Aug); 6) footer date. Do NOT index: retention (cl 2.12(5) — not subject to annual increase, stays $45.00), shift % (a % of earnings — self-indexes; only change if the certified % changes), qualification (cl 4.2 — no indexation clause, hold pending certified text), in-charge/laundry (move with the award/SWC, not the EBA). YEARS 2-3: each 1 Aug, agreement ladder × 1.025 applied to the PRECEDING AGREEMENT rate (offer wording), NOT the award. After each 1 Sep SWC the award ladder moves independently — keep BOTH ladders live and re-check the MAX winner per row. Caution: if an SWC is ever a flat dollar amount or tiered (not a flat %), the winning ladder can differ by classification — don't assume a blanket MAX. If certification lands after 1 Aug, the first rise backdates and arrives lump-sum-taxed — use the 'Other taxable earnings' row and point to the Pay Guide lump-sum explainer.</t>
   </si>
   <si>
     <t xml:space="preserve">State Wage Case 2026</t>

</xml_diff>

<commit_message>
Rename Excel 'Pay Notes' sheet to 'Pay Guide' (#16)
Renames the workbook tab (and its print-area/print-title references) and
the two in-sheet mentions that point readers to it, done via direct XML
edit so all formatting, formulas and protection are preserved untouched.
Also updates the workbook description on the calculator page.


Claude-Session: https://claude.ai/code/session_01FxBSYkNTAwxShAqXto2QT4

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PayCalc_V19.xlsx
+++ b/PayCalc_V19.xlsx
@@ -9,15 +9,15 @@
   </bookViews>
   <sheets>
     <sheet name="Pay Calculator" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Pay Notes" sheetId="2" state="visible" r:id="rId4"/>
+    <sheet name="Pay Guide" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Settings &amp; Rates" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="Tax Engine" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Area" vbProcedure="false">'Pay Calculator'!$A$1:$J$99</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Pay Calculator'!$1:$2</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Pay Notes'!$A$1:$J$51</definedName>
-    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'Pay Notes'!$1:$2</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'Pay Guide'!$A$1:$J$51</definedName>
+    <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Titles" vbProcedure="false">'Pay Guide'!$1:$2</definedName>
     <definedName function="false" hidden="false" name="BaseRate" vbProcedure="false">'Tax Engine'!$F$5</definedName>
     <definedName function="false" hidden="false" name="ConcCap" vbProcedure="false">'Settings &amp; Rates'!$B$44</definedName>
     <definedName function="false" hidden="false" name="ContribTax" vbProcedure="false">'Settings &amp; Rates'!$B$42</definedName>
@@ -528,7 +528,7 @@
     <t xml:space="preserve">Leave the payslip column blank when you are not reconciling. A mismatch usually means a rate on Settings &amp; Rates is stale, or payroll treats an allowance differently — see block E for the clause each rate comes from.</t>
   </si>
   <si>
-    <t xml:space="preserve">PayCalc V19 · pay scale award 01.09.2025 · tax tables ATO 01.07.2026 · plain-English guide on the Pay Notes tab · rates, sources &amp; incoming changes on Settings &amp; Rates</t>
+    <t xml:space="preserve">PayCalc V19 · pay scale award 01.09.2025 · tax tables ATO 01.07.2026 · plain-English guide on the Pay Guide tab · rates, sources &amp; incoming changes on Settings &amp; Rates</t>
   </si>
   <si>
     <t xml:space="preserve">PAY  NOTES</t>
@@ -1023,7 +1023,7 @@
     <t xml:space="preserve">OFFER 16.07.2026 — not yet certified</t>
   </si>
   <si>
-    <t xml:space="preserve">Employer Offer dated 16.07.2026 (3-year term, expires 31.07.2029). Three increases: 1 Aug 2026 = 3.5% (3% + 0.5% CPI uplift, already triggered), 1 Aug 2027 = 2.5%, 1 Aug 2028 = 2.5%. The FIRST rise applies to the higher of Award or Agreement — i.e. the Award rate (cl 2.18(6) retained). Allowances that track wages rise by the same %. CONDITIONAL: all unions must agree in-principle by 31.08.2026 to hold the 1 Aug date, else it shifts to the first of the month agreement is reached. NOT applied yet — do not change rates until certified. When certified, the EBA rise builds a SEPARATE agreement ladder — it must NOT be added to block A. Block A is the AWARD ladder; it moves only at a State Wage Case / reprint (~1 Sep). The certification (~1 Aug) and the SWC (~1 Sep) are only 31 days apart, so bumping block A on certification would be overwritten a month later = double-bump. Correct method: 1) build an Agreement-rate column = (award rate at 31.07.2026) × the agreed % for each row; 2) operational rate + $379 cap × same %; 3) set pay = MAX(award, agreement) per row (cl 2.18(6)); 4) block A itself changes ONLY at the SWC/reprint; 5) pull the Rates-checked-until tripwire back to the first-rise date (1 Aug if unions agree by 31 Aug); 6) footer date. Do NOT index: retention (cl 2.12(5) — not subject to annual increase, stays $45.00), shift % (a % of earnings — self-indexes; only change if the certified % changes), qualification (cl 4.2 — no indexation clause, hold pending certified text), in-charge/laundry (move with the award/SWC, not the EBA). YEARS 2-3: each 1 Aug, agreement ladder × 1.025 applied to the PRECEDING AGREEMENT rate (offer wording), NOT the award. After each 1 Sep SWC the award ladder moves independently — keep BOTH ladders live and re-check the MAX winner per row. Caution: if an SWC is ever a flat dollar amount or tiered (not a flat %), the winning ladder can differ by classification — don't assume a blanket MAX. If certification lands after 1 Aug, the first rise backdates and arrives lump-sum-taxed — use the 'Other taxable earnings' row and point to the Pay Notes lump-sum explainer.</t>
+    <t xml:space="preserve">Employer Offer dated 16.07.2026 (3-year term, expires 31.07.2029). Three increases: 1 Aug 2026 = 3.5% (3% + 0.5% CPI uplift, already triggered), 1 Aug 2027 = 2.5%, 1 Aug 2028 = 2.5%. The FIRST rise applies to the higher of Award or Agreement — i.e. the Award rate (cl 2.18(6) retained). Allowances that track wages rise by the same %. CONDITIONAL: all unions must agree in-principle by 31.08.2026 to hold the 1 Aug date, else it shifts to the first of the month agreement is reached. NOT applied yet — do not change rates until certified. When certified, the EBA rise builds a SEPARATE agreement ladder — it must NOT be added to block A. Block A is the AWARD ladder; it moves only at a State Wage Case / reprint (~1 Sep). The certification (~1 Aug) and the SWC (~1 Sep) are only 31 days apart, so bumping block A on certification would be overwritten a month later = double-bump. Correct method: 1) build an Agreement-rate column = (award rate at 31.07.2026) × the agreed % for each row; 2) operational rate + $379 cap × same %; 3) set pay = MAX(award, agreement) per row (cl 2.18(6)); 4) block A itself changes ONLY at the SWC/reprint; 5) pull the Rates-checked-until tripwire back to the first-rise date (1 Aug if unions agree by 31 Aug); 6) footer date. Do NOT index: retention (cl 2.12(5) — not subject to annual increase, stays $45.00), shift % (a % of earnings — self-indexes; only change if the certified % changes), qualification (cl 4.2 — no indexation clause, hold pending certified text), in-charge/laundry (move with the award/SWC, not the EBA). YEARS 2-3: each 1 Aug, agreement ladder × 1.025 applied to the PRECEDING AGREEMENT rate (offer wording), NOT the award. After each 1 Sep SWC the award ladder moves independently — keep BOTH ladders live and re-check the MAX winner per row. Caution: if an SWC is ever a flat dollar amount or tiered (not a flat %), the winning ladder can differ by classification — don't assume a blanket MAX. If certification lands after 1 Aug, the first rise backdates and arrives lump-sum-taxed — use the 'Other taxable earnings' row and point to the Pay Guide lump-sum explainer.</t>
   </si>
   <si>
     <t xml:space="preserve">State Wage Case 2026</t>

</xml_diff>